<commit_message>
hardware: swap pots to RK09K1130A70, clear enclosure fit hold
Switch RV1-RV6 on CONTROL board BOM from RK09K1130A5R (20mm shaft,
C209779) to RK09K1130A70 (30mm shaft, C351173) - same ALPS drawing-7
footprint, no board rework. Fixes knob protrusion (2.75mm -> 12.75mm
past the face) that was blocking the PCBWay order.

Updates ENCLOSURE_FIT.md and fab/README_PCBWAY.md hold notices to
reflect the fix. Fab package is cleared to order.
</commit_message>
<xml_diff>
--- a/hardware/BOM.xlsx
+++ b/hardware/BOM.xlsx
@@ -4994,7 +4994,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>RK09K1130A5R</t>
+          <t>RK09K1130A70</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -5004,12 +5004,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>C209779</t>
+          <t>C351173</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>GENUINE ALPS B10k linear snap-in, 3.4k stock</t>
+          <t>GENUINE ALPS B10k linear snap-in, 30mm shaft (was A5R/20mm - fixes knob protrusion, same footprint), JLC 7.7k stock</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
@@ -5038,7 +5038,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>RK09K1130A5R</t>
+          <t>RK09K1130A70</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -5048,12 +5048,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>C209779</t>
+          <t>C351173</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>GENUINE ALPS B10k linear snap-in, 3.4k stock</t>
+          <t>GENUINE ALPS B10k linear snap-in, 30mm shaft (was A5R/20mm - fixes knob protrusion, same footprint), JLC 7.7k stock</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>RK09K1130A5R</t>
+          <t>RK09K1130A70</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -5092,12 +5092,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>C209779</t>
+          <t>C351173</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>GENUINE ALPS B10k linear snap-in, 3.4k stock</t>
+          <t>GENUINE ALPS B10k linear snap-in, 30mm shaft (was A5R/20mm - fixes knob protrusion, same footprint), JLC 7.7k stock</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>RK09K1130A5R</t>
+          <t>RK09K1130A70</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -5136,12 +5136,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>C209779</t>
+          <t>C351173</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>GENUINE ALPS B10k linear snap-in, 3.4k stock</t>
+          <t>GENUINE ALPS B10k linear snap-in, 30mm shaft (was A5R/20mm - fixes knob protrusion, same footprint), JLC 7.7k stock</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
@@ -5170,7 +5170,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>RK09K1130A5R</t>
+          <t>RK09K1130A70</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -5180,12 +5180,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>C209779</t>
+          <t>C351173</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>GENUINE ALPS B10k linear snap-in, 3.4k stock</t>
+          <t>GENUINE ALPS B10k linear snap-in, 30mm shaft (was A5R/20mm - fixes knob protrusion, same footprint), JLC 7.7k stock</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>RK09K1130A5R</t>
+          <t>RK09K1130A70</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -5224,12 +5224,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>C209779</t>
+          <t>C351173</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>GENUINE ALPS B10k linear snap-in, 3.4k stock</t>
+          <t>GENUINE ALPS B10k linear snap-in, 30mm shaft (was A5R/20mm - fixes knob protrusion, same footprint), JLC 7.7k stock</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
@@ -5397,7 +5397,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Pots: RK09K1130A5R C209779 genuine ALPS. Jacks: C309273 / C5146694 / C319095 all verified.</t>
+          <t xml:space="preserve">  Pots: RK09K1130A70 C351173 genuine ALPS (30mm shaft - fixes knob protrusion, drop-in same footprint). Jacks: C309273 / C5146694 / C319095 all verified.</t>
         </is>
       </c>
     </row>

</xml_diff>